<commit_message>
module PDFs get the heatmaps too, all twelve rows labelled
</commit_message>
<xml_diff>
--- a/04_Network/02_Contrasts/c_data/02_contrasts.xlsx
+++ b/04_Network/02_Contrasts/c_data/02_contrasts.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1407" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1488" uniqueCount="221">
   <si>
     <t>sheet</t>
   </si>
@@ -293,6 +293,15 @@
     <t>0dc36d2d3fb0960d7b9f4242bb0d9080</t>
   </si>
   <si>
+    <t>phenotype</t>
+  </si>
+  <si>
+    <t>00_Input/phenotype.csv</t>
+  </si>
+  <si>
+    <t>5a1989db406daa0b70189a9f0df52cf3</t>
+  </si>
+  <si>
     <t>package</t>
   </si>
   <si>
@@ -302,6 +311,15 @@
     <t>source</t>
   </si>
   <si>
+    <t>BiocGenerics</t>
+  </si>
+  <si>
+    <t>0.58.0</t>
+  </si>
+  <si>
+    <t>Bioconductor 3.23 (R 4.6.0)</t>
+  </si>
+  <si>
     <t>BiocManager</t>
   </si>
   <si>
@@ -311,12 +329,78 @@
     <t>CRAN (R 4.6.0)</t>
   </si>
   <si>
+    <t>bit</t>
+  </si>
+  <si>
+    <t>4.6.0</t>
+  </si>
+  <si>
+    <t>bit64</t>
+  </si>
+  <si>
+    <t>4.8.0</t>
+  </si>
+  <si>
+    <t>circlize</t>
+  </si>
+  <si>
+    <t>0.4.18</t>
+  </si>
+  <si>
     <t>cli</t>
   </si>
   <si>
     <t>3.6.6</t>
   </si>
   <si>
+    <t>clue</t>
+  </si>
+  <si>
+    <t>0.3-68</t>
+  </si>
+  <si>
+    <t>cluster</t>
+  </si>
+  <si>
+    <t>2.1.8.2</t>
+  </si>
+  <si>
+    <t>codetools</t>
+  </si>
+  <si>
+    <t>0.2-20</t>
+  </si>
+  <si>
+    <t>colorspace</t>
+  </si>
+  <si>
+    <t>2.1-2</t>
+  </si>
+  <si>
+    <t>ComplexHeatmap</t>
+  </si>
+  <si>
+    <t>2.28.0</t>
+  </si>
+  <si>
+    <t>crayon</t>
+  </si>
+  <si>
+    <t>1.5.3</t>
+  </si>
+  <si>
+    <t>digest</t>
+  </si>
+  <si>
+    <t>0.6.39</t>
+  </si>
+  <si>
+    <t>doParallel</t>
+  </si>
+  <si>
+    <t>1.0.17</t>
+  </si>
+  <si>
     <t>dplyr</t>
   </si>
   <si>
@@ -329,18 +413,33 @@
     <t>2.1.2</t>
   </si>
   <si>
+    <t>foreach</t>
+  </si>
+  <si>
+    <t>1.5.2</t>
+  </si>
+  <si>
     <t>generics</t>
   </si>
   <si>
     <t>0.1.4</t>
   </si>
   <si>
+    <t>GetoptLong</t>
+  </si>
+  <si>
+    <t>1.1.1</t>
+  </si>
+  <si>
     <t>ggplot2</t>
   </si>
   <si>
     <t>4.0.3</t>
   </si>
   <si>
+    <t>GlobalOptions</t>
+  </si>
+  <si>
     <t>glue</t>
   </si>
   <si>
@@ -359,6 +458,24 @@
     <t>1.0.2</t>
   </si>
   <si>
+    <t>hms</t>
+  </si>
+  <si>
+    <t>1.1.4</t>
+  </si>
+  <si>
+    <t>IRanges</t>
+  </si>
+  <si>
+    <t>2.46.0</t>
+  </si>
+  <si>
+    <t>iterators</t>
+  </si>
+  <si>
+    <t>1.0.14</t>
+  </si>
+  <si>
     <t>labeling</t>
   </si>
   <si>
@@ -383,9 +500,6 @@
     <t>3.68.1</t>
   </si>
   <si>
-    <t>Bioconductor 3.23 (R 4.6.0)</t>
-  </si>
-  <si>
     <t>magrittr</t>
   </si>
   <si>
@@ -398,6 +512,12 @@
     <t>1.7-5</t>
   </si>
   <si>
+    <t>matrixStats</t>
+  </si>
+  <si>
+    <t>1.5.0</t>
+  </si>
+  <si>
     <t>mgcv</t>
   </si>
   <si>
@@ -422,6 +542,12 @@
     <t>2.0.3</t>
   </si>
   <si>
+    <t>png</t>
+  </si>
+  <si>
+    <t>0.1-9</t>
+  </si>
+  <si>
     <t>purrr</t>
   </si>
   <si>
@@ -440,12 +566,24 @@
     <t>1.1-3</t>
   </si>
   <si>
+    <t>readr</t>
+  </si>
+  <si>
+    <t>2.2.0</t>
+  </si>
+  <si>
     <t>renv</t>
   </si>
   <si>
     <t>1.2.3</t>
   </si>
   <si>
+    <t>rjson</t>
+  </si>
+  <si>
+    <t>0.2.23</t>
+  </si>
+  <si>
     <t>rlang</t>
   </si>
   <si>
@@ -461,6 +599,12 @@
     <t>2.1.1</t>
   </si>
   <si>
+    <t>S4Vectors</t>
+  </si>
+  <si>
+    <t>0.50.0</t>
+  </si>
+  <si>
     <t>S7</t>
   </si>
   <si>
@@ -479,6 +623,12 @@
     <t>1.2.4</t>
   </si>
   <si>
+    <t>shape</t>
+  </si>
+  <si>
+    <t>1.4.6.1</t>
+  </si>
+  <si>
     <t>statmod</t>
   </si>
   <si>
@@ -512,10 +662,22 @@
     <t>tidyselect</t>
   </si>
   <si>
+    <t>tzdb</t>
+  </si>
+  <si>
+    <t>0.5.0</t>
+  </si>
+  <si>
     <t>vctrs</t>
   </si>
   <si>
     <t>0.7.3</t>
+  </si>
+  <si>
+    <t>vroom</t>
+  </si>
+  <si>
+    <t>1.7.1</t>
   </si>
   <si>
     <t>withr</t>
@@ -11322,7 +11484,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -11389,6 +11551,17 @@
       </c>
       <c r="C6" t="s">
         <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -11398,414 +11571,700 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C3" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B4" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C5" t="s">
         <v>101</v>
-      </c>
-      <c r="C5" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B6" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C6" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B7" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C7" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B8" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B9" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C9" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B10" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C10" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B11" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C11" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B12" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C12" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B13" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C13" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B14" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C14" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B15" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C15" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B16" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C16" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B17" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C17" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B18" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C18" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B19" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C19" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B20" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C20" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B21" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C21" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B22" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C22" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B23" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C23" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B24" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C24" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B25" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C25" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B26" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C26" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B27" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C27" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B28" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C28" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B29" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C29" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B30" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C30" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B31" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C31" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B32" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C32" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B33" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C33" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B34" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C34" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B35" t="s">
-        <v>99</v>
+        <v>164</v>
       </c>
       <c r="C35" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B36" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C36" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B37" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C37" t="s">
-        <v>95</v>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>169</v>
+      </c>
+      <c r="B38" t="s">
+        <v>170</v>
+      </c>
+      <c r="C38" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>171</v>
+      </c>
+      <c r="B39" t="s">
+        <v>172</v>
+      </c>
+      <c r="C39" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>173</v>
+      </c>
+      <c r="B40" t="s">
+        <v>174</v>
+      </c>
+      <c r="C40" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>175</v>
+      </c>
+      <c r="B41" t="s">
+        <v>176</v>
+      </c>
+      <c r="C41" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>177</v>
+      </c>
+      <c r="B42" t="s">
+        <v>178</v>
+      </c>
+      <c r="C42" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>179</v>
+      </c>
+      <c r="B43" t="s">
+        <v>180</v>
+      </c>
+      <c r="C43" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>181</v>
+      </c>
+      <c r="B44" t="s">
+        <v>182</v>
+      </c>
+      <c r="C44" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>183</v>
+      </c>
+      <c r="B45" t="s">
+        <v>184</v>
+      </c>
+      <c r="C45" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
+        <v>185</v>
+      </c>
+      <c r="B46" t="s">
+        <v>186</v>
+      </c>
+      <c r="C46" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" t="s">
+        <v>187</v>
+      </c>
+      <c r="B47" t="s">
+        <v>188</v>
+      </c>
+      <c r="C47" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
+        <v>190</v>
+      </c>
+      <c r="B48" t="s">
+        <v>191</v>
+      </c>
+      <c r="C48" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" t="s">
+        <v>192</v>
+      </c>
+      <c r="B49" t="s">
+        <v>193</v>
+      </c>
+      <c r="C49" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
+        <v>194</v>
+      </c>
+      <c r="B50" t="s">
+        <v>195</v>
+      </c>
+      <c r="C50" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
+        <v>196</v>
+      </c>
+      <c r="B51" t="s">
+        <v>197</v>
+      </c>
+      <c r="C51" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
+        <v>198</v>
+      </c>
+      <c r="B52" t="s">
+        <v>199</v>
+      </c>
+      <c r="C52" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
+        <v>200</v>
+      </c>
+      <c r="B53" t="s">
+        <v>201</v>
+      </c>
+      <c r="C53" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
+        <v>202</v>
+      </c>
+      <c r="B54" t="s">
+        <v>203</v>
+      </c>
+      <c r="C54" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
+        <v>204</v>
+      </c>
+      <c r="B55" t="s">
+        <v>205</v>
+      </c>
+      <c r="C55" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
+        <v>206</v>
+      </c>
+      <c r="B56" t="s">
+        <v>207</v>
+      </c>
+      <c r="C56" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
+        <v>208</v>
+      </c>
+      <c r="B57" t="s">
+        <v>209</v>
+      </c>
+      <c r="C57" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
+        <v>210</v>
+      </c>
+      <c r="B58" t="s">
+        <v>211</v>
+      </c>
+      <c r="C58" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
+        <v>212</v>
+      </c>
+      <c r="B59" t="s">
+        <v>127</v>
+      </c>
+      <c r="C59" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
+        <v>213</v>
+      </c>
+      <c r="B60" t="s">
+        <v>214</v>
+      </c>
+      <c r="C60" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>215</v>
+      </c>
+      <c r="B61" t="s">
+        <v>216</v>
+      </c>
+      <c r="C61" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>217</v>
+      </c>
+      <c r="B62" t="s">
+        <v>218</v>
+      </c>
+      <c r="C62" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>219</v>
+      </c>
+      <c r="B63" t="s">
+        <v>220</v>
+      </c>
+      <c r="C63" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>